<commit_message>
Improve Excel export functionality with enhanced formatting and calculations
Update Excel export functions to include rounded quantities, subtotals, and a summary sheet.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 1b527f10-1a06-472b-80ce-a7cbcc7df77d
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: cf2a71b4-4920-4c07-9a01-e28570f23bdc
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/9263845a-7cc6-4b33-8ac4-ac779607e95a/1b527f10-1a06-472b-80ce-a7cbcc7df77d/UIUNImK
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/orders_2026-05-21.xlsx
+++ b/orders_2026-05-21.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="الطلبات التفصيلية" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="ملخص الكميات" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +26,69 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="001F4E79"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002E75B6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F7FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D6E4F0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +96,57 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BDD7EE"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BDD7EE"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BDD7EE"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BDD7EE"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,137 +512,270 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>Order Name</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Username</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Product</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Quantity</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Timestamp</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>تقرير الطلبات — 2026-05-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>الاسم</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>المستخدم</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>المنتج</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>الكمية (معدّلة)</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>الوقت</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  موارد</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>موارد</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Agjamp</t>
-        </is>
-      </c>
-      <c r="C2" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>@Agjamp</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>ماء</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>5</v>
-      </c>
-      <c r="E2" t="inlineStr">
+      <c r="D4" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>2026-05-21 06:30:50</t>
         </is>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>موارد</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>@Agjamp</t>
+        </is>
+      </c>
+      <c r="C5" s="7" t="inlineStr">
+        <is>
+          <t>عشاء</t>
+        </is>
+      </c>
+      <c r="D5" s="7" t="n">
+        <v>2</v>
+      </c>
+      <c r="E5" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-21 06:30:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>موارد</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>@Agjamp</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>غداء</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>2026-05-21 06:30:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>موارد</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>@Agjamp</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>فطور</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" s="7" t="inlineStr">
+        <is>
+          <t>2026-05-21 06:30:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>المجموع الفرعي</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n"/>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>ماء: 6  |  عشاء: 2  |  غداء: 6  |  فطور: 6</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="E8" s="9" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A8:B8"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A3:E3"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ملخص إجمالي للكميات</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>المنتج</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>الكمية الإجمالية</t>
+        </is>
+      </c>
+    </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>موارد</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Agjamp</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
+        <is>
+          <t>ماء</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>عشاء</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>2026-05-21 06:30:50</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>موارد</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Agjamp</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
+      <c r="B4" s="7" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>غداء</t>
         </is>
       </c>
-      <c r="D4" t="n">
-        <v>5</v>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>2026-05-21 06:30:50</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>موارد</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Agjamp</t>
-        </is>
-      </c>
-      <c r="C5" t="inlineStr">
+      <c r="B5" s="5" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>فطور</t>
         </is>
       </c>
-      <c r="D5" t="n">
-        <v>5</v>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>2026-05-21 06:30:50</t>
-        </is>
+      <c r="B6" s="7" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="11" t="inlineStr">
+        <is>
+          <t>الإجمالي الكلي</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>20</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:B1"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>